<commit_message>
mejora de servicio de sl JournalEntries
</commit_message>
<xml_diff>
--- a/assets/ASIENTOS_CONTABLES_CABECERA.xlsx
+++ b/assets/ASIENTOS_CONTABLES_CABECERA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\proyecto4\OneDrive - LLAMA GAS S.A\Documentos\GitHub\Jobs_JE\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34DEE9E4-20BC-4F15-AB20-DEE99A242B5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42222E46-6FE7-4F90-81E5-9C30040135C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-975" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28365" yWindow="3000" windowWidth="17280" windowHeight="8790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CabeceraSaldosBancosFinal" sheetId="4" r:id="rId1"/>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Cabecera_Saldos_Bancos!$A$2:$Q$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CabeceraSaldosBancosFinal!$A$2:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CabeceraSaldosBancosFinal!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="28">
   <si>
     <t>JdtNum</t>
   </si>
@@ -116,15 +116,6 @@
   </si>
   <si>
     <t>Saldos de Bancos al 30/06/2013 (USD)</t>
-  </si>
-  <si>
-    <t>Referencia 2</t>
-  </si>
-  <si>
-    <t>Referencia</t>
-  </si>
-  <si>
-    <t>Codigo proyecto</t>
   </si>
   <si>
     <t>Saldos de planillas Mes de Julio</t>
@@ -161,7 +152,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -188,12 +179,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="6" tint="-0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -211,7 +196,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -220,8 +205,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -526,7 +510,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="13.2"/>
   <cols>
     <col min="1" max="1" width="9.5546875" style="1" bestFit="1" customWidth="1"/>
@@ -542,81 +526,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="I1" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" s="8" t="s">
+      <c r="A2" s="6">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="I2" s="8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
-      <c r="A3" s="6">
-        <v>1</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>